<commit_message>
3_ml_model: remove amines 49-53, mark NMR-only reactants
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkLzRCnHQm67YFeR7F5Ysw
</commit_message>
<xml_diff>
--- a/3_ml_model/data/datasheets/PRISM_substrate_features.xlsx
+++ b/3_ml_model/data/datasheets/PRISM_substrate_features.xlsx
@@ -723,8 +723,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>0</v>
       </c>
@@ -899,8 +897,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>0</v>
       </c>
@@ -1075,8 +1071,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>0</v>
       </c>
@@ -1251,8 +1245,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>0</v>
       </c>
@@ -1427,8 +1419,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>0</v>
       </c>
@@ -1603,8 +1593,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>0</v>
       </c>
@@ -1779,8 +1767,6 @@
           <t>hetero</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>0</v>
       </c>
@@ -1955,8 +1941,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>0</v>
       </c>
@@ -2131,8 +2115,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>0</v>
       </c>
@@ -2307,8 +2289,6 @@
           <t>aliphatic</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>0</v>
       </c>
@@ -2663,8 +2643,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>0</v>
       </c>
@@ -3022,7 +3000,6 @@
       <c r="F15" t="n">
         <v>14.6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>3</v>
       </c>
@@ -3197,8 +3174,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>0</v>
       </c>
@@ -3373,8 +3348,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>0</v>
       </c>
@@ -3549,8 +3522,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>0</v>
       </c>
@@ -3725,8 +3696,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>0</v>
       </c>
@@ -3901,8 +3870,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>0</v>
       </c>
@@ -4077,8 +4044,6 @@
           <t>hetero</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>0</v>
       </c>
@@ -4613,8 +4578,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
         <v>0</v>
       </c>
@@ -4789,8 +4752,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>0</v>
       </c>
@@ -4968,7 +4929,6 @@
       <c r="F26" t="n">
         <v>14.9</v>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>2</v>
       </c>
@@ -5146,7 +5106,6 @@
       <c r="F27" t="n">
         <v>15.4</v>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>1</v>
       </c>
@@ -5324,7 +5283,6 @@
       <c r="F28" t="n">
         <v>18.4</v>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
         <v>1</v>
       </c>
@@ -5499,8 +5457,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
         <v>0</v>
       </c>
@@ -5675,8 +5631,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
         <v>0</v>
       </c>
@@ -5851,8 +5805,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
         <v>0</v>
       </c>
@@ -6027,8 +5979,6 @@
           <t>aliphatic</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
         <v>0</v>
       </c>
@@ -6206,7 +6156,6 @@
       <c r="F33" t="n">
         <v>10.9</v>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>2</v>
       </c>
@@ -6561,8 +6510,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
         <v>0</v>
       </c>
@@ -6920,7 +6867,6 @@
       <c r="F37" t="n">
         <v>14.4</v>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>1</v>
       </c>
@@ -7095,8 +7041,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
         <v>0</v>
       </c>
@@ -7271,8 +7215,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
         <v>0</v>
       </c>
@@ -7447,8 +7389,6 @@
           <t>aromatic</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
         <v>0</v>
       </c>
@@ -7626,7 +7566,6 @@
       <c r="F41" t="n">
         <v>11.9</v>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
         <v>2</v>
       </c>
@@ -7804,7 +7743,6 @@
       <c r="F42" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
         <v>2</v>
       </c>
@@ -8162,7 +8100,6 @@
       <c r="F44" t="n">
         <v>14.8</v>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
         <v>1</v>
       </c>
@@ -8337,8 +8274,6 @@
           <t>hetero</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
         <v>0</v>
       </c>
@@ -8696,7 +8631,6 @@
       <c r="F47" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
         <v>2</v>
       </c>
@@ -8858,7 +8792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO56"/>
+  <dimension ref="A1:AO51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13412,7 +13346,6 @@
           <t>2_aliphatic</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
         <v>7.5458</v>
       </c>
@@ -13503,10 +13436,6 @@
       <c r="AJ34" t="n">
         <v>-0.0135</v>
       </c>
-      <c r="AK34" t="inlineStr"/>
-      <c r="AL34" t="inlineStr"/>
-      <c r="AM34" t="inlineStr"/>
-      <c r="AN34" t="inlineStr"/>
       <c r="AO34" t="inlineStr">
         <is>
           <t>morfeus_amine</t>
@@ -15405,21 +15334,21 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>49_amine_pka.sdf</t>
+          <t>54_amine.sdf</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CCNCC</t>
+          <t>CNCCC(OC1=CC=C(C(F)(F)F)C=C1)C2=CC=CC=C2</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>train</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -15428,109 +15357,109 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>9.890000000000001</v>
+        <v>9.42</v>
       </c>
       <c r="G49" t="n">
-        <v>8.284730189742151</v>
+        <v>7.72592379900128</v>
       </c>
       <c r="H49" t="n">
-        <v>-4.18248479364823</v>
+        <v>4.46379355093466</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.348062649032318</v>
+        <v>-0.36872577067176</v>
       </c>
       <c r="J49" t="n">
-        <v>0.0368902727821491</v>
+        <v>-0.248385718513037</v>
       </c>
       <c r="K49" t="n">
-        <v>0.003993848855933</v>
+        <v>0.8314214076761099</v>
       </c>
       <c r="L49" t="n">
-        <v>-8.284730189742151</v>
+        <v>-7.72592379900128</v>
       </c>
       <c r="M49" t="n">
-        <v>12.4672149833903</v>
+        <v>3.26213024806661</v>
       </c>
       <c r="N49" t="n">
-        <v>79.3935764169872</v>
+        <v>84.5592995054681</v>
       </c>
       <c r="O49" t="n">
-        <v>249.850391218182</v>
+        <v>536.849929204428</v>
       </c>
       <c r="P49" t="n">
-        <v>334.678918856469</v>
+        <v>854.977257547653</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.722114285908388</v>
+        <v>0.745506396592365</v>
       </c>
       <c r="R49" t="n">
-        <v>13.8234874979268</v>
+        <v>18.5852509824437</v>
       </c>
       <c r="S49" t="n">
-        <v>17.5230853816876</v>
+        <v>24.1147153063105</v>
       </c>
       <c r="T49" t="n">
-        <v>-0.263094774003263</v>
+        <v>-0.258890996117932</v>
       </c>
       <c r="U49" t="n">
-        <v>0.200687489807115</v>
+        <v>-0.0075673347374361</v>
       </c>
       <c r="V49" t="n">
-        <v>0.208501130790826</v>
+        <v>0.114624150169128</v>
       </c>
       <c r="W49" t="n">
-        <v>71.5639341735435</v>
+        <v>43.2272393696937</v>
       </c>
       <c r="X49" t="n">
-        <v>4.6567659436115</v>
+        <v>3.55547848833296</v>
       </c>
       <c r="Y49" t="n">
-        <v>1.9934875629751</v>
+        <v>1.93594223095107</v>
       </c>
       <c r="Z49" t="n">
-        <v>4.38859421430796</v>
+        <v>7.67232482459937</v>
       </c>
       <c r="AA49" t="n">
-        <v>0.0224589669223451</v>
+        <v>-0.0261131870968252</v>
       </c>
       <c r="AB49" t="n">
-        <v>0.0064804209176421</v>
+        <v>-0.0064876442323584</v>
       </c>
       <c r="AC49" t="n">
-        <v>-0.0363272607032198</v>
+        <v>-0.0349437004408519</v>
       </c>
       <c r="AD49" t="n">
-        <v>71.7077460635346</v>
+        <v>65.3972803307244</v>
       </c>
       <c r="AE49" t="n">
-        <v>4.66001320840639</v>
+        <v>4.90488284391125</v>
       </c>
       <c r="AF49" t="n">
-        <v>1.9131474229072</v>
+        <v>1.95611558287542</v>
       </c>
       <c r="AG49" t="n">
-        <v>4.39135259505738</v>
+        <v>9.470493564734371</v>
       </c>
       <c r="AH49" t="n">
-        <v>0.0182295258009417</v>
+        <v>-0.005694565927417</v>
       </c>
       <c r="AI49" t="n">
-        <v>0.0010556928694416</v>
+        <v>-0.0057395633223811</v>
       </c>
       <c r="AJ49" t="n">
-        <v>-0.0322296352415084</v>
+        <v>-0.0304806705447599</v>
       </c>
       <c r="AK49" t="n">
-        <v>4.30015911397692</v>
+        <v>4.55333575540073</v>
       </c>
       <c r="AL49" t="n">
-        <v>1062.74035808026</v>
+        <v>1093.57795898278</v>
       </c>
       <c r="AM49" t="n">
-        <v>4.29651933897355</v>
+        <v>4.47607419660747</v>
       </c>
       <c r="AN49" t="n">
-        <v>1062.29040098284</v>
+        <v>1084.21989697196</v>
       </c>
       <c r="AO49" t="inlineStr">
         <is>
@@ -15540,21 +15469,21 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>50_amine_pka.sdf</t>
+          <t>55_amine.sdf</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CCCCC(CC)CNCC(CC)CCCC</t>
+          <t>FC(C=C1)=CC=C1[C@H]2[C@H](COC3=CC4=C(OCO4)C=C3)CNCC2</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>train</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -15563,109 +15492,109 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>9.68</v>
+        <v>9.31</v>
       </c>
       <c r="G50" t="n">
-        <v>7.46662871493331</v>
+        <v>7.12643523316406</v>
       </c>
       <c r="H50" t="n">
-        <v>-2.65650409616274</v>
+        <v>4.44207532734405</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.344031829015225</v>
+        <v>-0.362716617257703</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0111444203903569</v>
+        <v>-0.246451498693595</v>
       </c>
       <c r="K50" t="n">
-        <v>1.07474744412296e-05</v>
+        <v>0.750165808828329</v>
       </c>
       <c r="L50" t="n">
-        <v>-7.46662871493331</v>
+        <v>-7.12643523316406</v>
       </c>
       <c r="M50" t="n">
-        <v>10.123132811096</v>
+        <v>2.68435990582001</v>
       </c>
       <c r="N50" t="n">
-        <v>98.0933057344504</v>
+        <v>77.4837545179051</v>
       </c>
       <c r="O50" t="n">
-        <v>567.450845268851</v>
+        <v>534.349136443977</v>
       </c>
       <c r="P50" t="n">
-        <v>902.172784888866</v>
+        <v>881.11689552435</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.749058568310742</v>
+        <v>0.749423184402664</v>
       </c>
       <c r="R50" t="n">
-        <v>17.0420783407513</v>
+        <v>19.4380281341531</v>
       </c>
       <c r="S50" t="n">
-        <v>24.2860451683676</v>
+        <v>18.389157541215</v>
       </c>
       <c r="T50" t="n">
-        <v>-0.272305435642365</v>
+        <v>-0.255641652595125</v>
       </c>
       <c r="U50" t="n">
-        <v>0.0901237126105171</v>
+        <v>0.0106362106994484</v>
       </c>
       <c r="V50" t="n">
-        <v>0.133875643173702</v>
+        <v>0.100817381226451</v>
       </c>
       <c r="W50" t="n">
-        <v>97.8537935685742</v>
+        <v>90.7604682018851</v>
       </c>
       <c r="X50" t="n">
-        <v>6.98178529963607</v>
+        <v>7.03472233586782</v>
       </c>
       <c r="Y50" t="n">
-        <v>2.36908308784755</v>
+        <v>1.7</v>
       </c>
       <c r="Z50" t="n">
-        <v>8.432307551020591</v>
+        <v>9.07001496196993</v>
       </c>
       <c r="AA50" t="n">
-        <v>0.0168520772729173</v>
+        <v>0.0072746251062648</v>
       </c>
       <c r="AB50" t="n">
-        <v>0.0109706478642698</v>
+        <v>-0.0061707526627179</v>
       </c>
       <c r="AC50" t="n">
-        <v>-0.0283338009041616</v>
+        <v>-0.0158330734927004</v>
       </c>
       <c r="AD50" t="n">
-        <v>95.90736500658539</v>
+        <v>82.19921565263201</v>
       </c>
       <c r="AE50" t="n">
-        <v>8.16390426273249</v>
+        <v>6.29486309990811</v>
       </c>
       <c r="AF50" t="n">
-        <v>2.38843497100166</v>
+        <v>1.7</v>
       </c>
       <c r="AG50" t="n">
-        <v>7.74815147684763</v>
+        <v>9.312344106431439</v>
       </c>
       <c r="AH50" t="n">
-        <v>0.0160243690411715</v>
+        <v>0.0079554384067572</v>
       </c>
       <c r="AI50" t="n">
-        <v>0.0099786416632263</v>
+        <v>-0.0067026768124254</v>
       </c>
       <c r="AJ50" t="n">
-        <v>-0.0276372661199847</v>
+        <v>-0.0156463855621073</v>
       </c>
       <c r="AK50" t="n">
-        <v>4.22741027636143</v>
+        <v>4.39480329626071</v>
       </c>
       <c r="AL50" t="n">
-        <v>1053.71244661622</v>
+        <v>1074.37187653333</v>
       </c>
       <c r="AM50" t="n">
-        <v>4.2193348754846</v>
+        <v>4.37773799479624</v>
       </c>
       <c r="AN50" t="n">
-        <v>1052.70505761048</v>
+        <v>1072.28188358064</v>
       </c>
       <c r="AO50" t="inlineStr">
         <is>
@@ -15675,21 +15604,21 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>51_amine_pka.sdf</t>
+          <t>56_amine.sdf</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>C1CCNC1</t>
+          <t>C[C@@H](NCCCC1=CC(C(F)(F)F)=CC=C1)C2=CC=CC3=CC=CC=C32</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>train</t>
+          <t>test</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -15698,786 +15627,111 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>10.87</v>
+        <v>8.4</v>
       </c>
       <c r="G51" t="n">
-        <v>8.727133719208449</v>
+        <v>7.29605034984126</v>
       </c>
       <c r="H51" t="n">
-        <v>-4.09174786658198</v>
+        <v>5.33449582830429</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.358863622235436</v>
+        <v>-0.357848116037496</v>
       </c>
       <c r="J51" t="n">
-        <v>0.0347938946540723</v>
+        <v>-0.260499023975776</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0003138877471273</v>
+        <v>1.1127189471631</v>
       </c>
       <c r="L51" t="n">
-        <v>-8.727133719208449</v>
+        <v>-7.29605034984126</v>
       </c>
       <c r="M51" t="n">
-        <v>12.8188815857904</v>
+        <v>1.96155452153697</v>
       </c>
       <c r="N51" t="n">
-        <v>71.7846200556389</v>
+        <v>104.320622047229</v>
       </c>
       <c r="O51" t="n">
-        <v>228.470140536447</v>
+        <v>621.591248652786</v>
       </c>
       <c r="P51" t="n">
-        <v>299.83224427508</v>
+        <v>1001.76455758677</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.83293680244466</v>
+        <v>0.673571530808205</v>
       </c>
       <c r="R51" t="n">
-        <v>13.8655772776854</v>
+        <v>19.2135712431433</v>
       </c>
       <c r="S51" t="n">
-        <v>15.9009255897727</v>
+        <v>27.2067505030011</v>
       </c>
       <c r="T51" t="n">
-        <v>-0.263047602009537</v>
+        <v>-0.261217058136727</v>
       </c>
       <c r="U51" t="n">
-        <v>0.164215688359872</v>
+        <v>0.0044823906631223</v>
       </c>
       <c r="V51" t="n">
-        <v>0.213082307776983</v>
+        <v>0.09560728393655731</v>
       </c>
       <c r="W51" t="n">
-        <v>67.2359807133017</v>
+        <v>113.138644189157</v>
       </c>
       <c r="X51" t="n">
-        <v>4.2606239528633</v>
+        <v>8.48749735287177</v>
       </c>
       <c r="Y51" t="n">
-        <v>1.7</v>
+        <v>3.11566183539634</v>
       </c>
       <c r="Z51" t="n">
-        <v>4.23477771632087</v>
+        <v>6.35403008675662</v>
       </c>
       <c r="AA51" t="n">
-        <v>0.0124170618113185</v>
+        <v>0.0458739973182809</v>
       </c>
       <c r="AB51" t="n">
-        <v>0.008234879727124099</v>
+        <v>-0.0033407211985984</v>
       </c>
       <c r="AC51" t="n">
-        <v>-0.0340546447648043</v>
+        <v>-0.0086213237670234</v>
       </c>
       <c r="AD51" t="n">
-        <v>67.2427790935558</v>
+        <v>100.446591207032</v>
       </c>
       <c r="AE51" t="n">
-        <v>4.26062548319673</v>
+        <v>8.310086588914841</v>
       </c>
       <c r="AF51" t="n">
-        <v>1.7</v>
+        <v>3.52859128049643</v>
       </c>
       <c r="AG51" t="n">
-        <v>4.23475772903447</v>
+        <v>7.52646856482877</v>
       </c>
       <c r="AH51" t="n">
-        <v>0.0124063454537852</v>
+        <v>0.0318633095545976</v>
       </c>
       <c r="AI51" t="n">
-        <v>0.008309807881888001</v>
+        <v>-0.0044236315342191</v>
       </c>
       <c r="AJ51" t="n">
-        <v>-0.0340517689178274</v>
+        <v>-0.0142390333021736</v>
       </c>
       <c r="AK51" t="n">
-        <v>4.31211589009409</v>
+        <v>4.37407629212353</v>
       </c>
       <c r="AL51" t="n">
-        <v>1064.21682992716</v>
+        <v>1071.83537752451</v>
       </c>
       <c r="AM51" t="n">
-        <v>4.31126781567053</v>
+        <v>4.38468032030675</v>
       </c>
       <c r="AN51" t="n">
-        <v>1064.11216856521</v>
+        <v>1073.13302623119</v>
       </c>
       <c r="AO51" t="inlineStr">
-        <is>
-          <t>substrate_scope.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>52</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>52_amine_pka.sdf</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>C1CN(CCN1)C2=CC=CC=C2F</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>train</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2_aliphatic</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="G52" t="n">
-        <v>7.06117287996187</v>
-      </c>
-      <c r="H52" t="n">
-        <v>3.03998756316648</v>
-      </c>
-      <c r="I52" t="n">
-        <v>-0.34599862491521</v>
-      </c>
-      <c r="J52" t="n">
-        <v>-0.22367315284268</v>
-      </c>
-      <c r="K52" t="n">
-        <v>0.389310563278631</v>
-      </c>
-      <c r="L52" t="n">
-        <v>-7.06117287996187</v>
-      </c>
-      <c r="M52" t="n">
-        <v>4.02118531679539</v>
-      </c>
-      <c r="N52" t="n">
-        <v>74.72884165800249</v>
-      </c>
-      <c r="O52" t="n">
-        <v>361.890802813913</v>
-      </c>
-      <c r="P52" t="n">
-        <v>543.663011216176</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>0.767372974861721</v>
-      </c>
-      <c r="R52" t="n">
-        <v>17.3829641770483</v>
-      </c>
-      <c r="S52" t="n">
-        <v>17.5041448349511</v>
-      </c>
-      <c r="T52" t="n">
-        <v>-0.26365412757212</v>
-      </c>
-      <c r="U52" t="n">
-        <v>0.0116607700505714</v>
-      </c>
-      <c r="V52" t="n">
-        <v>0.0871811808751964</v>
-      </c>
-      <c r="W52" t="n">
-        <v>74.238312375051</v>
-      </c>
-      <c r="X52" t="n">
-        <v>6.5500511353302</v>
-      </c>
-      <c r="Y52" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="Z52" t="n">
-        <v>7.99937396523043</v>
-      </c>
-      <c r="AA52" t="n">
-        <v>0.005661312809152</v>
-      </c>
-      <c r="AB52" t="n">
-        <v>-0.0074310653537903</v>
-      </c>
-      <c r="AC52" t="n">
-        <v>-0.0190400055130243</v>
-      </c>
-      <c r="AD52" t="n">
-        <v>73.9564410706684</v>
-      </c>
-      <c r="AE52" t="n">
-        <v>6.5977745437387</v>
-      </c>
-      <c r="AF52" t="n">
-        <v>1.75251591933721</v>
-      </c>
-      <c r="AG52" t="n">
-        <v>7.97631430736128</v>
-      </c>
-      <c r="AH52" t="n">
-        <v>0.0096941267979175</v>
-      </c>
-      <c r="AI52" t="n">
-        <v>-0.0070921718987475</v>
-      </c>
-      <c r="AJ52" t="n">
-        <v>-0.0204835698350877</v>
-      </c>
-      <c r="AK52" t="n">
-        <v>3.95359091630186</v>
-      </c>
-      <c r="AL52" t="n">
-        <v>1019.01546656628</v>
-      </c>
-      <c r="AM52" t="n">
-        <v>4.01240210324444</v>
-      </c>
-      <c r="AN52" t="n">
-        <v>1026.53904232776</v>
-      </c>
-      <c r="AO52" t="inlineStr">
-        <is>
-          <t>substrate_scope.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>53</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>53_amine_pka.sdf</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>CNCC1=C2C=CC=CC2=CC3=CC=CC=C31</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>train</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2_aliphatic</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>9.41</v>
-      </c>
-      <c r="G53" t="n">
-        <v>6.86272182151267</v>
-      </c>
-      <c r="H53" t="n">
-        <v>5.479778811516</v>
-      </c>
-      <c r="I53" t="n">
-        <v>-0.352432178811398</v>
-      </c>
-      <c r="J53" t="n">
-        <v>-0.28444844598438</v>
-      </c>
-      <c r="K53" t="n">
-        <v>1.12774995795453</v>
-      </c>
-      <c r="L53" t="n">
-        <v>-6.86272182151267</v>
-      </c>
-      <c r="M53" t="n">
-        <v>1.38294300999667</v>
-      </c>
-      <c r="N53" t="n">
-        <v>84.8009034806532</v>
-      </c>
-      <c r="O53" t="n">
-        <v>431.513411519575</v>
-      </c>
-      <c r="P53" t="n">
-        <v>673.9956199505471</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>0.753439638668431</v>
-      </c>
-      <c r="R53" t="n">
-        <v>19.0884737028018</v>
-      </c>
-      <c r="S53" t="n">
-        <v>23.5686087947323</v>
-      </c>
-      <c r="T53" t="n">
-        <v>-0.253526422190653</v>
-      </c>
-      <c r="U53" t="n">
-        <v>0.0075814291342199</v>
-      </c>
-      <c r="V53" t="n">
-        <v>0.0789247354188941</v>
-      </c>
-      <c r="W53" t="n">
-        <v>41.514047545654</v>
-      </c>
-      <c r="X53" t="n">
-        <v>3.55418383294547</v>
-      </c>
-      <c r="Y53" t="n">
-        <v>2.00716942021907</v>
-      </c>
-      <c r="Z53" t="n">
-        <v>6.33318463897</v>
-      </c>
-      <c r="AA53" t="n">
-        <v>-0.0220089906724232</v>
-      </c>
-      <c r="AB53" t="n">
-        <v>-0.0126662209827938</v>
-      </c>
-      <c r="AC53" t="n">
-        <v>-0.0281511213203265</v>
-      </c>
-      <c r="AD53" t="n">
-        <v>69.0035595793743</v>
-      </c>
-      <c r="AE53" t="n">
-        <v>4.47165861439052</v>
-      </c>
-      <c r="AF53" t="n">
-        <v>2.509573290691</v>
-      </c>
-      <c r="AG53" t="n">
-        <v>6.79358604337647</v>
-      </c>
-      <c r="AH53" t="n">
-        <v>-0.0032603382520386</v>
-      </c>
-      <c r="AI53" t="n">
-        <v>-0.0119843811438743</v>
-      </c>
-      <c r="AJ53" t="n">
-        <v>-0.0250521578996683</v>
-      </c>
-      <c r="AK53" t="n">
-        <v>4.52266033993062</v>
-      </c>
-      <c r="AL53" t="n">
-        <v>1089.88806544154</v>
-      </c>
-      <c r="AM53" t="n">
-        <v>4.37556468079268</v>
-      </c>
-      <c r="AN53" t="n">
-        <v>1071.86622687027</v>
-      </c>
-      <c r="AO53" t="inlineStr">
-        <is>
-          <t>substrate_scope.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>54</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>54_amine.sdf</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>CNCCC(OC1=CC=C(C(F)(F)F)C=C1)C2=CC=CC=C2</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>2_aliphatic</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>9.42</v>
-      </c>
-      <c r="G54" t="n">
-        <v>7.72592379900128</v>
-      </c>
-      <c r="H54" t="n">
-        <v>4.46379355093466</v>
-      </c>
-      <c r="I54" t="n">
-        <v>-0.36872577067176</v>
-      </c>
-      <c r="J54" t="n">
-        <v>-0.248385718513037</v>
-      </c>
-      <c r="K54" t="n">
-        <v>0.8314214076761099</v>
-      </c>
-      <c r="L54" t="n">
-        <v>-7.72592379900128</v>
-      </c>
-      <c r="M54" t="n">
-        <v>3.26213024806661</v>
-      </c>
-      <c r="N54" t="n">
-        <v>84.5592995054681</v>
-      </c>
-      <c r="O54" t="n">
-        <v>536.849929204428</v>
-      </c>
-      <c r="P54" t="n">
-        <v>854.977257547653</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>0.745506396592365</v>
-      </c>
-      <c r="R54" t="n">
-        <v>18.5852509824437</v>
-      </c>
-      <c r="S54" t="n">
-        <v>24.1147153063105</v>
-      </c>
-      <c r="T54" t="n">
-        <v>-0.258890996117932</v>
-      </c>
-      <c r="U54" t="n">
-        <v>-0.0075673347374361</v>
-      </c>
-      <c r="V54" t="n">
-        <v>0.114624150169128</v>
-      </c>
-      <c r="W54" t="n">
-        <v>43.2272393696937</v>
-      </c>
-      <c r="X54" t="n">
-        <v>3.55547848833296</v>
-      </c>
-      <c r="Y54" t="n">
-        <v>1.93594223095107</v>
-      </c>
-      <c r="Z54" t="n">
-        <v>7.67232482459937</v>
-      </c>
-      <c r="AA54" t="n">
-        <v>-0.0261131870968252</v>
-      </c>
-      <c r="AB54" t="n">
-        <v>-0.0064876442323584</v>
-      </c>
-      <c r="AC54" t="n">
-        <v>-0.0349437004408519</v>
-      </c>
-      <c r="AD54" t="n">
-        <v>65.3972803307244</v>
-      </c>
-      <c r="AE54" t="n">
-        <v>4.90488284391125</v>
-      </c>
-      <c r="AF54" t="n">
-        <v>1.95611558287542</v>
-      </c>
-      <c r="AG54" t="n">
-        <v>9.470493564734371</v>
-      </c>
-      <c r="AH54" t="n">
-        <v>-0.005694565927417</v>
-      </c>
-      <c r="AI54" t="n">
-        <v>-0.0057395633223811</v>
-      </c>
-      <c r="AJ54" t="n">
-        <v>-0.0304806705447599</v>
-      </c>
-      <c r="AK54" t="n">
-        <v>4.55333575540073</v>
-      </c>
-      <c r="AL54" t="n">
-        <v>1093.57795898278</v>
-      </c>
-      <c r="AM54" t="n">
-        <v>4.47607419660747</v>
-      </c>
-      <c r="AN54" t="n">
-        <v>1084.21989697196</v>
-      </c>
-      <c r="AO54" t="inlineStr">
-        <is>
-          <t>substrate_scope.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>55</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>55_amine.sdf</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>FC(C=C1)=CC=C1[C@H]2[C@H](COC3=CC4=C(OCO4)C=C3)CNCC2</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>2_aliphatic</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>9.31</v>
-      </c>
-      <c r="G55" t="n">
-        <v>7.12643523316406</v>
-      </c>
-      <c r="H55" t="n">
-        <v>4.44207532734405</v>
-      </c>
-      <c r="I55" t="n">
-        <v>-0.362716617257703</v>
-      </c>
-      <c r="J55" t="n">
-        <v>-0.246451498693595</v>
-      </c>
-      <c r="K55" t="n">
-        <v>0.750165808828329</v>
-      </c>
-      <c r="L55" t="n">
-        <v>-7.12643523316406</v>
-      </c>
-      <c r="M55" t="n">
-        <v>2.68435990582001</v>
-      </c>
-      <c r="N55" t="n">
-        <v>77.4837545179051</v>
-      </c>
-      <c r="O55" t="n">
-        <v>534.349136443977</v>
-      </c>
-      <c r="P55" t="n">
-        <v>881.11689552435</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>0.749423184402664</v>
-      </c>
-      <c r="R55" t="n">
-        <v>19.4380281341531</v>
-      </c>
-      <c r="S55" t="n">
-        <v>18.389157541215</v>
-      </c>
-      <c r="T55" t="n">
-        <v>-0.255641652595125</v>
-      </c>
-      <c r="U55" t="n">
-        <v>0.0106362106994484</v>
-      </c>
-      <c r="V55" t="n">
-        <v>0.100817381226451</v>
-      </c>
-      <c r="W55" t="n">
-        <v>90.7604682018851</v>
-      </c>
-      <c r="X55" t="n">
-        <v>7.03472233586782</v>
-      </c>
-      <c r="Y55" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="Z55" t="n">
-        <v>9.07001496196993</v>
-      </c>
-      <c r="AA55" t="n">
-        <v>0.0072746251062648</v>
-      </c>
-      <c r="AB55" t="n">
-        <v>-0.0061707526627179</v>
-      </c>
-      <c r="AC55" t="n">
-        <v>-0.0158330734927004</v>
-      </c>
-      <c r="AD55" t="n">
-        <v>82.19921565263201</v>
-      </c>
-      <c r="AE55" t="n">
-        <v>6.29486309990811</v>
-      </c>
-      <c r="AF55" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="AG55" t="n">
-        <v>9.312344106431439</v>
-      </c>
-      <c r="AH55" t="n">
-        <v>0.0079554384067572</v>
-      </c>
-      <c r="AI55" t="n">
-        <v>-0.0067026768124254</v>
-      </c>
-      <c r="AJ55" t="n">
-        <v>-0.0156463855621073</v>
-      </c>
-      <c r="AK55" t="n">
-        <v>4.39480329626071</v>
-      </c>
-      <c r="AL55" t="n">
-        <v>1074.37187653333</v>
-      </c>
-      <c r="AM55" t="n">
-        <v>4.37773799479624</v>
-      </c>
-      <c r="AN55" t="n">
-        <v>1072.28188358064</v>
-      </c>
-      <c r="AO55" t="inlineStr">
-        <is>
-          <t>substrate_scope.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>56</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>56_amine.sdf</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>C[C@@H](NCCCC1=CC(C(F)(F)F)=CC=C1)C2=CC=CC3=CC=CC=C32</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2_aliphatic</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G56" t="n">
-        <v>7.29605034984126</v>
-      </c>
-      <c r="H56" t="n">
-        <v>5.33449582830429</v>
-      </c>
-      <c r="I56" t="n">
-        <v>-0.357848116037496</v>
-      </c>
-      <c r="J56" t="n">
-        <v>-0.260499023975776</v>
-      </c>
-      <c r="K56" t="n">
-        <v>1.1127189471631</v>
-      </c>
-      <c r="L56" t="n">
-        <v>-7.29605034984126</v>
-      </c>
-      <c r="M56" t="n">
-        <v>1.96155452153697</v>
-      </c>
-      <c r="N56" t="n">
-        <v>104.320622047229</v>
-      </c>
-      <c r="O56" t="n">
-        <v>621.591248652786</v>
-      </c>
-      <c r="P56" t="n">
-        <v>1001.76455758677</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>0.673571530808205</v>
-      </c>
-      <c r="R56" t="n">
-        <v>19.2135712431433</v>
-      </c>
-      <c r="S56" t="n">
-        <v>27.2067505030011</v>
-      </c>
-      <c r="T56" t="n">
-        <v>-0.261217058136727</v>
-      </c>
-      <c r="U56" t="n">
-        <v>0.0044823906631223</v>
-      </c>
-      <c r="V56" t="n">
-        <v>0.09560728393655731</v>
-      </c>
-      <c r="W56" t="n">
-        <v>113.138644189157</v>
-      </c>
-      <c r="X56" t="n">
-        <v>8.48749735287177</v>
-      </c>
-      <c r="Y56" t="n">
-        <v>3.11566183539634</v>
-      </c>
-      <c r="Z56" t="n">
-        <v>6.35403008675662</v>
-      </c>
-      <c r="AA56" t="n">
-        <v>0.0458739973182809</v>
-      </c>
-      <c r="AB56" t="n">
-        <v>-0.0033407211985984</v>
-      </c>
-      <c r="AC56" t="n">
-        <v>-0.0086213237670234</v>
-      </c>
-      <c r="AD56" t="n">
-        <v>100.446591207032</v>
-      </c>
-      <c r="AE56" t="n">
-        <v>8.310086588914841</v>
-      </c>
-      <c r="AF56" t="n">
-        <v>3.52859128049643</v>
-      </c>
-      <c r="AG56" t="n">
-        <v>7.52646856482877</v>
-      </c>
-      <c r="AH56" t="n">
-        <v>0.0318633095545976</v>
-      </c>
-      <c r="AI56" t="n">
-        <v>-0.0044236315342191</v>
-      </c>
-      <c r="AJ56" t="n">
-        <v>-0.0142390333021736</v>
-      </c>
-      <c r="AK56" t="n">
-        <v>4.37407629212353</v>
-      </c>
-      <c r="AL56" t="n">
-        <v>1071.83537752451</v>
-      </c>
-      <c r="AM56" t="n">
-        <v>4.38468032030675</v>
-      </c>
-      <c r="AN56" t="n">
-        <v>1073.13302623119</v>
-      </c>
-      <c r="AO56" t="inlineStr">
         <is>
           <t>substrate_scope.xlsx</t>
         </is>

</xml_diff>